<commit_message>
paper run 2026-09-29 10:20
</commit_message>
<xml_diff>
--- a/reports/2026-09-29.xlsx
+++ b/reports/2026-09-29.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,49 @@
       </c>
       <c r="K5" t="n">
         <v>3.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-29T10:12:04.995093+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00123</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-9.279999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -699,7 +742,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -709,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66.63</v>
+        <v>57.35</v>
       </c>
     </row>
     <row r="7">
@@ -739,7 +782,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-4.48</v>
+        <v>-13.76</v>
       </c>
     </row>
     <row r="9">
@@ -749,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15.87</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2181.82</v>
+        <v>2172.54</v>
       </c>
     </row>
     <row r="12">
@@ -810,16 +853,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
         <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>398.84</v>
+        <v>184.05</v>
       </c>
       <c r="E15" t="n">
-        <v>8.300000000000001</v>
+        <v>-0.98</v>
       </c>
     </row>
     <row r="16">
@@ -874,16 +917,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
         <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>304.81</v>
+        <v>90.02</v>
       </c>
       <c r="E19" t="n">
-        <v>12.78</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="20">
@@ -919,16 +962,16 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>-100.68</v>
+        <v>-315.47</v>
       </c>
       <c r="E22" t="n">
-        <v>-4.48</v>
+        <v>-13.76</v>
       </c>
     </row>
     <row r="23">
@@ -983,13 +1026,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" t="n">
         <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>340.33</v>
+        <v>231.24</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -1002,16 +1045,16 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>140.46</v>
+        <v>34.76</v>
       </c>
       <c r="E27" t="n">
-        <v>66.63</v>
+        <v>57.35</v>
       </c>
     </row>
     <row r="29">
@@ -1066,13 +1109,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
         <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>12.78</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="35">
@@ -1104,13 +1147,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" t="n">
         <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>8.300000000000001</v>
+        <v>-0.98</v>
       </c>
     </row>
     <row r="37">
@@ -1199,182 +1242,198 @@
         <v>62.13</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-9.279999999999999</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>2</v>
-      </c>
-      <c r="C45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" t="n">
-        <v>67.31</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>-4.48</v>
+        <v>67.31</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-13.76</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>0.60–0.62</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B48" t="n">
         <v>1</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C48" t="n">
         <v>1</v>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
         <v>3.8</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" t="n">
-        <v>67.31</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>2</v>
       </c>
       <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>67.31</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
         <v>1</v>
       </c>
-      <c r="D51" t="n">
-        <v>-0.68</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="D52" t="n">
+        <v>-9.960000000000001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>1</v>
-      </c>
-      <c r="C54" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" t="n">
-        <v>-4.48</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-4.48</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B56" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" t="n">
         <v>3</v>
       </c>
-      <c r="C55" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" t="n">
-        <v>71.11</v>
+      <c r="D56" t="n">
+        <v>61.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-29 17:56
</commit_message>
<xml_diff>
--- a/reports/2026-09-29.xlsx
+++ b/reports/2026-09-29.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +687,307 @@
       </c>
       <c r="K6" t="n">
         <v>-9.279999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-29T13:26:51.326191+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00142</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-5.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-29T14:38:50.185295+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>45.06</v>
+      </c>
+      <c r="G8" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00116</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>35.41</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-29T16:13:00.006685+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F9" t="n">
+        <v>57.93</v>
+      </c>
+      <c r="G9" t="n">
+        <v>99.88</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.00132</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>41.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-29T16:13:50.101121+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>45.76</v>
+      </c>
+      <c r="G10" t="n">
+        <v>88</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-0.00122</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>42.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-29T16:57:57.998997+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F11" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G11" t="n">
+        <v>90</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.00104</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>44.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:33:55.930314+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>18</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.00202</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>8.640000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-29T17:43:28.021798+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-0.00123</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +1023,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -732,7 +1033,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -742,7 +1043,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -752,7 +1053,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
@@ -762,7 +1063,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57.35</v>
+        <v>224.89</v>
       </c>
     </row>
     <row r="7">
@@ -772,7 +1073,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>71.11</v>
+        <v>244.55</v>
       </c>
     </row>
     <row r="8">
@@ -782,7 +1083,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-13.76</v>
+        <v>-19.66</v>
       </c>
     </row>
     <row r="9">
@@ -792,7 +1093,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.17</v>
+        <v>12.44</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +1103,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2172.54</v>
+        <v>2340.079999999999</v>
       </c>
     </row>
     <row r="12">
@@ -853,16 +1154,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C15" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D15" t="n">
-        <v>184.05</v>
+        <v>637.87</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.98</v>
+        <v>80.27</v>
       </c>
     </row>
     <row r="16">
@@ -872,16 +1173,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>182.48</v>
+        <v>832.7</v>
       </c>
       <c r="E16" t="n">
-        <v>58.33</v>
+        <v>144.62</v>
       </c>
     </row>
     <row r="17">
@@ -894,288 +1195,304 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>276.51</v>
+        <v>169.52</v>
       </c>
       <c r="E18" t="n">
-        <v>53.85</v>
+        <v>41.95</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>90.02</v>
+        <v>203.62</v>
       </c>
       <c r="E19" t="n">
-        <v>3.5</v>
+        <v>44.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>11</v>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="n">
+        <v>777.4</v>
+      </c>
+      <c r="E20" t="n">
+        <v>90.36</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>577.15</v>
+        <v>320.03</v>
       </c>
       <c r="E21" t="n">
-        <v>67.31</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-315.47</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-13.76</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D23" t="n">
-        <v>104.85</v>
+        <v>1373.76</v>
       </c>
       <c r="E23" t="n">
-        <v>3.8</v>
+        <v>162.29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-95.95999999999999</v>
+      </c>
+      <c r="E24" t="n">
+        <v>57.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D25" t="n">
-        <v>100.53</v>
+        <v>192.77</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>5</v>
-      </c>
-      <c r="C26" t="n">
-        <v>4</v>
-      </c>
-      <c r="D26" t="n">
-        <v>231.24</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>34.76</v>
+        <v>184.37</v>
       </c>
       <c r="E27" t="n">
-        <v>57.35</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" t="n">
+        <v>803.11</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>12</v>
+      </c>
+      <c r="C29" t="n">
+        <v>9</v>
+      </c>
+      <c r="D29" t="n">
+        <v>483.09</v>
+      </c>
+      <c r="E29" t="n">
+        <v>224.89</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>53.85</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>XRP</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>3</v>
-      </c>
-      <c r="C33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" t="n">
-        <v>3.5</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>41.95</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>44.1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>4</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.98</v>
+        <v>90.36</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>58.33</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1197,93 +1514,93 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>00</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D40" t="n">
-        <v>8.98</v>
+        <v>80.27</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>-4.48</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" t="n">
-        <v>62.13</v>
+        <v>144.62</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
         <v>1</v>
       </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-9.279999999999999</v>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8.98</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-4.48</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1293,67 +1610,77 @@
         <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>67.31</v>
+        <v>62.13</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>-13.76</v>
+        <v>-9.279999999999999</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>1</v>
       </c>
       <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-5.9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
         <v>1</v>
       </c>
-      <c r="D48" t="n">
-        <v>3.8</v>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>35.41</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>128.29</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1363,77 +1690,201 @@
         <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>67.31</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>3</v>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="n">
-        <v>-9.960000000000001</v>
+        <v>9.74</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" t="n">
+        <v>5</v>
+      </c>
+      <c r="D54" t="n">
+        <v>162.29</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>-4.48</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" t="n">
+        <v>146.82</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="n">
+        <v>69.43000000000001</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>8.640000000000001</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D64" t="n">
+        <v>89.45</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>4</v>
-      </c>
-      <c r="C56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" t="n">
-        <v>61.83</v>
+      <c r="B65" t="n">
+        <v>7</v>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="n">
+        <v>135.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-30 03:38
</commit_message>
<xml_diff>
--- a/reports/2026-09-29.xlsx
+++ b/reports/2026-09-29.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -988,6 +988,49 @@
       </c>
       <c r="K13" t="n">
         <v>1.1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29T22:41:33.355377+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F14" t="n">
+        <v>48.98</v>
+      </c>
+      <c r="G14" t="n">
+        <v>87.45999999999999</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.00105</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>38.48</v>
       </c>
     </row>
   </sheetData>
@@ -1001,7 +1044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1023,7 +1066,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -1033,7 +1076,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1053,7 +1096,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.7692307692307693</v>
       </c>
     </row>
     <row r="6">
@@ -1063,7 +1106,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>224.89</v>
+        <v>263.37</v>
       </c>
     </row>
     <row r="7">
@@ -1073,7 +1116,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>244.55</v>
+        <v>283.03</v>
       </c>
     </row>
     <row r="8">
@@ -1093,7 +1136,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12.44</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="10">
@@ -1103,7 +1146,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2340.079999999999</v>
+        <v>2377.519999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1154,16 +1197,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>637.87</v>
+        <v>724.7</v>
       </c>
       <c r="E15" t="n">
-        <v>80.27</v>
+        <v>118.75</v>
       </c>
     </row>
     <row r="16">
@@ -1237,16 +1280,16 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>12</v>
+      </c>
+      <c r="C20" t="n">
         <v>11</v>
       </c>
-      <c r="C20" t="n">
-        <v>10</v>
-      </c>
       <c r="D20" t="n">
-        <v>777.4</v>
+        <v>864.23</v>
       </c>
       <c r="E20" t="n">
-        <v>90.36</v>
+        <v>128.84</v>
       </c>
     </row>
     <row r="21">
@@ -1301,16 +1344,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>-95.95999999999999</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>57.7</v>
+        <v>96.18000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1384,16 +1427,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>483.09</v>
+        <v>569.92</v>
       </c>
       <c r="E29" t="n">
-        <v>224.89</v>
+        <v>263.37</v>
       </c>
     </row>
     <row r="31">
@@ -1464,13 +1507,13 @@
         </is>
       </c>
       <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="n">
         <v>4</v>
       </c>
-      <c r="C36" t="n">
-        <v>3</v>
-      </c>
       <c r="D36" t="n">
-        <v>90.36</v>
+        <v>128.84</v>
       </c>
     </row>
     <row r="37">
@@ -1518,13 +1561,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D40" t="n">
-        <v>80.27</v>
+        <v>118.75</v>
       </c>
     </row>
     <row r="41">
@@ -1693,198 +1736,214 @@
         <v>9.74</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>38.48</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>5</v>
-      </c>
-      <c r="C54" t="n">
-        <v>5</v>
-      </c>
-      <c r="D54" t="n">
-        <v>162.29</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>5</v>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D55" t="n">
-        <v>57.7</v>
+        <v>162.29</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>6</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>96.18000000000001</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>0.60–0.62</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B57" t="n">
         <v>2</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C57" t="n">
         <v>2</v>
       </c>
-      <c r="D56" t="n">
+      <c r="D57" t="n">
         <v>4.9</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" t="n">
-        <v>4</v>
-      </c>
-      <c r="D59" t="n">
-        <v>146.82</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D60" t="n">
-        <v>69.43000000000001</v>
+        <v>185.3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>7</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>69.43000000000001</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>0.20%+</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="B62" t="n">
         <v>1</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C62" t="n">
         <v>1</v>
       </c>
-      <c r="D61" t="n">
+      <c r="D62" t="n">
         <v>8.640000000000001</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>5</v>
-      </c>
-      <c r="C64" t="n">
-        <v>4</v>
-      </c>
-      <c r="D64" t="n">
-        <v>89.45</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" t="n">
+        <v>4</v>
+      </c>
+      <c r="D65" t="n">
+        <v>89.45</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B65" t="n">
-        <v>7</v>
-      </c>
-      <c r="C65" t="n">
-        <v>5</v>
-      </c>
-      <c r="D65" t="n">
-        <v>135.44</v>
+      <c r="B66" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" t="n">
+        <v>6</v>
+      </c>
+      <c r="D66" t="n">
+        <v>173.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>